<commit_message>
feat: AmanahOS mobile friendly
</commit_message>
<xml_diff>
--- a/docs/pageCast info FINAL.xlsx
+++ b/docs/pageCast info FINAL.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Documents\00 StoryBook\pageCast\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A349F084-A2D1-4F9B-85E6-88FDF3DDAABB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4150D67-80E5-4C43-A2DA-339265BDFA33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Info" sheetId="1" r:id="rId1"/>
@@ -28,12 +28,12 @@
     <sheet name="HH-S5" sheetId="13" r:id="rId13"/>
     <sheet name="KAC-P1" sheetId="14" r:id="rId14"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1715" uniqueCount="638">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1745" uniqueCount="668">
   <si>
     <t>pageCast Studio — Series &amp; Production Tracker</t>
   </si>
@@ -2004,12 +2004,669 @@
   <si>
     <t>sk_bfc7f43b9817c4561f939806cae357b9a0a6e2a2e1174972</t>
   </si>
+  <si>
+    <t>Workflow Guide</t>
+  </si>
+  <si>
+    <t>Complete pageCast production reference — skills, scripts, ComfyUI workflows and all command options.</t>
+  </si>
+  <si>
+    <t>Stage</t>
+  </si>
+  <si>
+    <t>Skills / Scripts / Options</t>
+  </si>
+  <si>
+    <t>Output</t>
+  </si>
+  <si>
+    <t>Write / Import Story</t>
+  </si>
+  <si>
+    <t>Scene &amp; Character Image Prompts</t>
+  </si>
+  <si>
+    <t>Character Prompts &amp; Images</t>
+  </si>
+  <si>
+    <t>Scene Images</t>
+  </si>
+  <si>
+    <t>SFX &amp; Ambience</t>
+  </si>
+  <si>
+    <t>Voice</t>
+  </si>
+  <si>
+    <t>pageCast Documents (DOCX + PDF)</t>
+  </si>
+  <si>
+    <t>Review &amp; QA</t>
+  </si>
+  <si>
+    <t>All production tabs in one window</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">*_pagecast.txt
+*_manuscript.docx
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t>saved inside .casts/&lt;book&gt;/</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">storybook-writer.skill
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Write original chapters in the style of a chosen master: Dahl, Rowling, Gaiman, Tolkien, Hemingway, and more
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t xml:space="preserve">storybook-importer.skill
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Convert any uploaded PDF or TXT manuscript into page
+Cast .txt import format
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t xml:space="preserve">castlet-writer.skill
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Write a new self-contained Castlet unit for an existing pageCast Collection using the Collection Story Bible
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t xml:space="preserve">hidden-heroes-writer.skill
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t>Write a new episode for the Hidden Heroes / Pahlawan Tersembunyi Indonesia series (Bahasa Indonesia, 6-phase structure)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">*_image_prompts.txt
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t>[Ch1Sc1] scene blocks
+[cover] book cover block
+[char:Name] character portrait blocks</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">storybook-image-prompt.skill
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t>Writes a visual prompt for every scene, a [cover] block, AND a [char:Name] portrait prompt block for every character found in the script. Run BEFORE generating images or character portraits.
+Output includes: scene prompts, cover prompt, character portrait prompts — all in one *_image_prompts.txt file</t>
+    </r>
+  </si>
+  <si>
+    <t>CHARACTER_REFS/Name.png
+CHARACTER_REFS/Name.prompt.txt</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">(Characters tab auto-generate)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">The app analyses [DIALOGUE]/[THOUGHT] tags and scene context to pre-fill a ComfyUI portrait prompt for each character. Click ✎ to refine and save to CHARACTER_REFS/Name.prompt.txt
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t xml:space="preserve">storybook-image-prompt.skill
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Also generates [char:Name] blocks in the image prompts file — copy the prompt= value into ComfyUI as the positive prompt.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t xml:space="preserve">ComfyUI: character_portrait_gen.json
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Set positive prompt = character prompt text. Set Save Image output path to .casts/&lt;book&gt;/CHARACTER_REFS/ so portrait saves as CharacterName.png automatically.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t xml:space="preserve">ComfyUI: character_reference_sheet.json
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Multi-pose reference sheet for visual consistency across all scenes.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t xml:space="preserve">ComfyUI: img2img_face_fix.json
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t>Img2img pass to fix and sharpen face details on existing portraits.</t>
+    </r>
+  </si>
+  <si>
+    <t>images/*.jpg
+cover.jpg</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">scene-image-producer.skill
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Generate all scene images via Pollinations.ai — free, no GPU needed. Uses *_image_prompts.txt automatically.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t xml:space="preserve">python skills/generate_images.py --folder .casts/&lt;book&gt; --style-pick 2--backend pollinations|hf|comfyui
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">└ Image backend: pollinations (default, free), hf (HuggingFace), comfyui (local GPU)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t xml:space="preserve">--style-pick 1-6
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">└ Pick a visual style preset by number — skips the interactive menu
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t xml:space="preserve">--overwrite
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">└ Regenerate images that already exist (default: skip existing)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t xml:space="preserve">--comfyui-url URL
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">└ ComfyUI server URL (default: http://localhost:8000)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t xml:space="preserve">--hf-token hf_...
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">└ HuggingFace API token (required for --backend hf)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t xml:space="preserve">--width W --height H
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">└ Output image dimensions in pixels
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t xml:space="preserve">--force-workflow NAME
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">└ Force a specific ComfyUI workflow JSON by name
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t xml:space="preserve">ComfyUI: scene_single_character.json
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Scene with one character reference.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t xml:space="preserve">ComfyUI: scene_dual_character.json
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Scene with two character references.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t xml:space="preserve">ComfyUI: txt2img_juggernaut.json
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t>General text-to-image for backgrounds and scenery.</t>
+    </r>
+  </si>
+  <si>
+    <t>sfx/*.mp3
+ambience/*.mp3</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">SFX tab ▶ Generate button
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t>Paste ElevenLabs API key, set durations, click Generate. Live SSE log. Skips files that already exist.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t xml:space="preserve">python scripts/generate_elevenlabs_audio.py --folder .casts/&lt;book&gt; --api-key sk_xxx--file path/to/file.txt
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">└ Process a single pagecast .txt file instead of whole folder
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t xml:space="preserve">--sfx-duration SEC
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">└ SFX clip length in seconds (default: 5)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t xml:space="preserve">--ambience-duration SEC
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t>└ Ambience clip length in seconds (default: 10)</t>
+    </r>
+  </si>
+  <si>
+    <t>Supabase Storage + blocks.audio_url
+Local voice/ folder is fallback only</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">python skills/voice_producer.py --book "Title" --gemini-key KEY
+--chapter N
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">└ Generate voice for a specific chapter onl
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t xml:space="preserve">--scene N
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t>└ Generate voice for a specific scene only
+Generates narration, dialogue and thought lines. Uploads to Supabase Storage and writes audio_url to blocks table.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">*_manuscript.docx
+*_PageCast.docx
+*_PageCast.pdf
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t>Visible in Manuscripts tab</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Writing skills auto-produce *_manuscript.docx alongside *_pagecast.txt — clean Word chapter text.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t xml:space="preserve">python skills/storybook_pdf.py --book "Title"
+--chapter N
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">└ Process a single chapter only (default: all chapters)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t xml:space="preserve">--out-dir PATH
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">└ Output directory (default: same as .casts/&lt;book&gt;/)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t xml:space="preserve">--no-pdf
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">└ Build *_PageCast.docx only — skip PDF conversion
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t xml:space="preserve">--pdf-from file.docx
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">└ Convert an existing .docx directly to PDF (use after manual editing with --no-pdf)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t xml:space="preserve">pdf (Cowork skill)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t>Merge, split or extract pages from PDF files.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">python skills/pageCast_gui.py
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t>All-in-one review GUI — Images, SFX, Voice, Script, Characters, Manuscripts, Dashboard, Workflow Guide</t>
+    </r>
+  </si>
+  <si>
+    <t>python skills/pageCast_gui.py</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="42">
+  <fonts count="47">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2272,6 +2929,30 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="14"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Arial Unicode MS"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="16">
     <fill>
@@ -2357,7 +3038,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="12">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -2480,11 +3161,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF30363D"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4"/>
   </cellStyleXfs>
-  <cellXfs count="109">
+  <cellXfs count="117">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
@@ -2716,18 +3406,73 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="4" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="4" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="37" fillId="12" borderId="4" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="30" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="30" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="37" fillId="12" borderId="4" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -2737,42 +3482,9 @@
     <xf numFmtId="0" fontId="38" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="29" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="30" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="30" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3054,7 +3766,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:F189"/>
+  <dimension ref="A2:F191"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="13.140625" customWidth="1"/>
@@ -3078,655 +3790,663 @@
         <v>45</v>
       </c>
     </row>
-    <row r="5" spans="1:4">
-      <c r="B5" s="6" t="s">
+    <row r="5" spans="1:4" s="115" customFormat="1">
+      <c r="B5" s="116" t="s">
+        <v>667</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" s="115" customFormat="1">
+      <c r="B6" s="116"/>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="B7" s="6" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="6" spans="1:4" s="9" customFormat="1">
-      <c r="B6" s="8" t="s">
+    <row r="8" spans="1:4" s="9" customFormat="1">
+      <c r="B8" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="C6" s="9" t="s">
+      <c r="C8" s="9" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="8" spans="1:4">
-      <c r="B8" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="C8" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4">
-      <c r="B9" s="10"/>
     </row>
     <row r="10" spans="1:4">
       <c r="B10" s="4" t="s">
-        <v>51</v>
+        <v>49</v>
+      </c>
+      <c r="C10" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="11" spans="1:4">
-      <c r="A11" t="s">
-        <v>52</v>
-      </c>
-      <c r="B11" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="C11" t="s">
-        <v>48</v>
-      </c>
+      <c r="B11" s="10"/>
     </row>
     <row r="12" spans="1:4">
       <c r="B12" s="4" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4">
+      <c r="A13" t="s">
+        <v>52</v>
+      </c>
+      <c r="B13" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="C13" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
+      <c r="B14" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C14" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="13" spans="1:4">
-      <c r="B13" s="10" t="s">
+    <row r="15" spans="1:4">
+      <c r="B15" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C15" t="s">
         <v>55</v>
       </c>
-      <c r="D13" t="s">
+      <c r="D15" t="s">
         <v>56</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4">
-      <c r="B14" s="10" t="s">
-        <v>57</v>
-      </c>
-      <c r="C14" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4">
-      <c r="B15" s="11" t="s">
-        <v>59</v>
-      </c>
-      <c r="C15" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="16" spans="1:4">
       <c r="B16" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C16" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="17" spans="2:5">
+      <c r="B17" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="C17" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="18" spans="2:5">
+      <c r="B18" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C18" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="17" spans="2:5">
-      <c r="B17" s="10"/>
-    </row>
-    <row r="18" spans="2:5">
-      <c r="B18" t="s">
-        <v>63</v>
-      </c>
-      <c r="C18" t="s">
-        <v>64</v>
-      </c>
-    </row>
     <row r="19" spans="2:5">
-      <c r="B19" t="s">
-        <v>65</v>
-      </c>
+      <c r="B19" s="10"/>
     </row>
     <row r="20" spans="2:5">
       <c r="B20" t="s">
-        <v>66</v>
+        <v>63</v>
+      </c>
+      <c r="C20" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="21" spans="2:5">
       <c r="B21" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="22" spans="2:5">
       <c r="B22" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="23" spans="2:5">
+      <c r="B23" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="24" spans="2:5">
+      <c r="B24" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="24" spans="2:5">
-      <c r="B24" s="10" t="s">
+    <row r="26" spans="2:5">
+      <c r="B26" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="C24" t="s">
+      <c r="C26" t="s">
         <v>70</v>
       </c>
-      <c r="D24" t="s">
+      <c r="D26" t="s">
         <v>71</v>
       </c>
-      <c r="E24" t="s">
+      <c r="E26" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="25" spans="2:5">
-      <c r="B25" s="10"/>
-    </row>
-    <row r="26" spans="2:5" ht="30" customHeight="1">
-      <c r="B26" s="5" t="s">
+    <row r="27" spans="2:5">
+      <c r="B27" s="10"/>
+    </row>
+    <row r="28" spans="2:5" ht="30" customHeight="1">
+      <c r="B28" s="5" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="27" spans="2:5">
-      <c r="B27" s="5"/>
-    </row>
-    <row r="28" spans="2:5">
-      <c r="B28" s="5"/>
     </row>
     <row r="29" spans="2:5">
       <c r="B29" s="5"/>
     </row>
     <row r="30" spans="2:5">
-      <c r="B30" s="4" t="s">
+      <c r="B30" s="5"/>
+    </row>
+    <row r="31" spans="2:5">
+      <c r="B31" s="5"/>
+    </row>
+    <row r="32" spans="2:5">
+      <c r="B32" s="4" t="s">
         <v>74</v>
-      </c>
-    </row>
-    <row r="31" spans="2:5">
-      <c r="B31" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="C31" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="32" spans="2:5">
-      <c r="B32" s="10" t="s">
-        <v>75</v>
-      </c>
-      <c r="C32" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="33" spans="1:3">
       <c r="B33" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="C33" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3">
+      <c r="B34" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="C34" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3">
+      <c r="B35" s="10" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="34" spans="1:3">
-      <c r="B34" s="10"/>
-    </row>
-    <row r="35" spans="1:3">
-      <c r="B35" s="4" t="s">
+    <row r="36" spans="1:3">
+      <c r="B36" s="10"/>
+    </row>
+    <row r="37" spans="1:3">
+      <c r="B37" s="4" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="36" spans="1:3">
-      <c r="A36" t="s">
+    <row r="38" spans="1:3">
+      <c r="A38" t="s">
         <v>79</v>
       </c>
-      <c r="B36" s="15" t="s">
+      <c r="B38" s="15" t="s">
         <v>80</v>
       </c>
-      <c r="C36" t="s">
+      <c r="C38" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="37" spans="1:3">
-      <c r="B37" s="15" t="s">
+    <row r="39" spans="1:3">
+      <c r="B39" s="15" t="s">
         <v>82</v>
       </c>
-      <c r="C37" t="s">
+      <c r="C39" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="38" spans="1:3">
-      <c r="B38" s="15" t="s">
+    <row r="40" spans="1:3">
+      <c r="B40" s="15" t="s">
         <v>84</v>
       </c>
-      <c r="C38" t="s">
+      <c r="C40" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="39" spans="1:3">
-      <c r="B39" s="4"/>
-    </row>
-    <row r="40" spans="1:3">
-      <c r="B40" s="4" t="s">
+    <row r="41" spans="1:3">
+      <c r="B41" s="4"/>
+    </row>
+    <row r="42" spans="1:3">
+      <c r="B42" s="4" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="41" spans="1:3">
-      <c r="B41" s="10" t="s">
+    <row r="43" spans="1:3">
+      <c r="B43" s="10" t="s">
         <v>87</v>
       </c>
-      <c r="C41" t="s">
+      <c r="C43" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="42" spans="1:3">
-      <c r="B42" s="10" t="s">
+    <row r="44" spans="1:3">
+      <c r="B44" s="10" t="s">
         <v>89</v>
       </c>
-      <c r="C42" t="s">
+      <c r="C44" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="44" spans="1:3">
-      <c r="B44" s="7" t="s">
+    <row r="46" spans="1:3">
+      <c r="B46" s="7" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="49" spans="1:2" s="9" customFormat="1">
-      <c r="A49" s="8" t="s">
+    <row r="51" spans="1:2" s="9" customFormat="1">
+      <c r="A51" s="8" t="s">
         <v>92</v>
       </c>
-      <c r="B49" s="8"/>
-    </row>
-    <row r="50" spans="1:2">
-      <c r="B50" s="6" t="s">
+      <c r="B51" s="8"/>
+    </row>
+    <row r="52" spans="1:2">
+      <c r="B52" s="6" t="s">
         <v>93</v>
-      </c>
-    </row>
-    <row r="53" spans="1:2">
-      <c r="B53" s="6" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="54" spans="1:2">
-      <c r="B54" s="6" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="55" spans="1:2">
       <c r="B55" s="6" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="56" spans="1:2">
       <c r="B56" s="6" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="57" spans="1:2">
       <c r="B57" s="6" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="58" spans="1:2">
       <c r="B58" s="6" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
     </row>
     <row r="59" spans="1:2">
       <c r="B59" s="6" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="60" spans="1:2">
       <c r="B60" s="6" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="61" spans="1:2">
       <c r="B61" s="6" t="s">
-        <v>102</v>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2">
+      <c r="B62" s="6" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="63" spans="1:2">
       <c r="B63" s="6" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="65" spans="2:2">
+      <c r="B65" s="6" t="s">
         <v>103</v>
-      </c>
-    </row>
-    <row r="64" spans="1:2">
-      <c r="B64" s="6" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="66" spans="2:2">
       <c r="B66" s="6" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="67" spans="2:2">
-      <c r="B67" s="6" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="68" spans="2:2">
       <c r="B68" s="6" t="s">
-        <v>107</v>
+        <v>105</v>
+      </c>
+    </row>
+    <row r="69" spans="2:2">
+      <c r="B69" s="6" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="70" spans="2:2">
       <c r="B70" s="6" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="71" spans="2:2">
-      <c r="B71" s="6" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="72" spans="2:2">
       <c r="B72" s="6" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
     </row>
     <row r="73" spans="2:2">
       <c r="B73" s="6" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="74" spans="2:2">
       <c r="B74" s="6" t="s">
-        <v>107</v>
+        <v>110</v>
+      </c>
+    </row>
+    <row r="75" spans="2:2">
+      <c r="B75" s="6" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="76" spans="2:2">
       <c r="B76" s="6" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
     </row>
     <row r="78" spans="2:2">
       <c r="B78" s="6" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="80" spans="2:2">
+      <c r="B80" s="6" t="s">
         <v>113</v>
-      </c>
-    </row>
-    <row r="79" spans="2:2">
-      <c r="B79" s="6" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="81" spans="1:2">
       <c r="B81" s="6" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="82" spans="1:2">
-      <c r="B82" s="6" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
     </row>
     <row r="83" spans="1:2">
       <c r="B83" s="6" t="s">
-        <v>117</v>
+        <v>115</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2">
+      <c r="B84" s="6" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="85" spans="1:2">
       <c r="B85" s="6" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="86" spans="1:2">
-      <c r="B86" s="6" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
     </row>
     <row r="87" spans="1:2">
       <c r="B87" s="6" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="88" spans="1:2">
       <c r="B88" s="6" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="89" spans="1:2">
       <c r="B89" s="6" t="s">
-        <v>117</v>
+        <v>120</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2">
+      <c r="B90" s="6" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="91" spans="1:2">
       <c r="B91" s="6" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="93" spans="1:2">
+      <c r="B93" s="6" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="94" spans="1:2" s="9" customFormat="1">
-      <c r="A94" s="9" t="s">
+    <row r="96" spans="1:2" s="9" customFormat="1">
+      <c r="A96" s="9" t="s">
         <v>123</v>
       </c>
-      <c r="B94" s="8"/>
-    </row>
-    <row r="95" spans="1:2">
-      <c r="B95" s="6" t="s">
+      <c r="B96" s="8"/>
+    </row>
+    <row r="97" spans="1:2">
+      <c r="B97" s="6" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="96" spans="1:2">
-      <c r="A96" t="s">
+    <row r="98" spans="1:2">
+      <c r="A98" t="s">
         <v>125</v>
       </c>
-      <c r="B96" s="6" t="s">
+      <c r="B98" s="6" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="98" spans="1:3">
-      <c r="B98" s="26" t="s">
+    <row r="100" spans="1:2">
+      <c r="B100" s="26" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="99" spans="1:3">
-      <c r="B99" s="26" t="s">
+    <row r="101" spans="1:2">
+      <c r="B101" s="26" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="103" spans="1:3">
-      <c r="B103" s="27" t="s">
+    <row r="105" spans="1:2">
+      <c r="B105" s="27" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="104" spans="1:3" ht="16.5" customHeight="1">
-      <c r="B104" s="28" t="s">
+    <row r="106" spans="1:2" ht="16.5" customHeight="1">
+      <c r="B106" s="28" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="105" spans="1:3" ht="16.5" customHeight="1">
-      <c r="B105" s="28" t="s">
+    <row r="107" spans="1:2" ht="16.5" customHeight="1">
+      <c r="B107" s="28" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="106" spans="1:3" ht="16.5" customHeight="1">
-      <c r="B106" s="28" t="s">
+    <row r="108" spans="1:2" ht="16.5" customHeight="1">
+      <c r="B108" s="28" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="107" spans="1:3" ht="16.5" customHeight="1">
-      <c r="B107" s="29" t="s">
+    <row r="109" spans="1:2" ht="16.5" customHeight="1">
+      <c r="B109" s="29" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="111" spans="1:3" s="9" customFormat="1">
-      <c r="A111" s="9" t="s">
+    <row r="113" spans="1:6" s="9" customFormat="1">
+      <c r="A113" s="9" t="s">
         <v>134</v>
       </c>
-      <c r="B111" s="9" t="s">
+      <c r="B113" s="9" t="s">
         <v>135</v>
       </c>
-      <c r="C111" s="9" t="s">
+      <c r="C113" s="9" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="113" spans="1:6" ht="16.5" customHeight="1">
-      <c r="B113" s="31" t="s">
+    <row r="115" spans="1:6" ht="16.5" customHeight="1">
+      <c r="B115" s="31" t="s">
         <v>137</v>
       </c>
-      <c r="C113" s="31" t="s">
+      <c r="C115" s="31" t="s">
         <v>138</v>
       </c>
-      <c r="D113" s="38"/>
-      <c r="E113" s="38"/>
-      <c r="F113" s="38"/>
-    </row>
-    <row r="114" spans="1:6" ht="16.5" customHeight="1">
-      <c r="B114" s="31" t="s">
+      <c r="D115" s="38"/>
+      <c r="E115" s="38"/>
+      <c r="F115" s="38"/>
+    </row>
+    <row r="116" spans="1:6" ht="16.5" customHeight="1">
+      <c r="B116" s="31" t="s">
         <v>139</v>
       </c>
-      <c r="C114" s="31" t="s">
+      <c r="C116" s="31" t="s">
         <v>140</v>
       </c>
-      <c r="D114" s="29"/>
-      <c r="E114" s="29"/>
-      <c r="F114" s="12"/>
-    </row>
-    <row r="115" spans="1:6">
-      <c r="B115" s="31" t="s">
-        <v>141</v>
-      </c>
-      <c r="C115" s="31" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="116" spans="1:6">
-      <c r="B116" s="31" t="s">
-        <v>143</v>
-      </c>
-      <c r="C116" s="31" t="s">
-        <v>144</v>
-      </c>
+      <c r="D116" s="29"/>
+      <c r="E116" s="29"/>
+      <c r="F116" s="12"/>
     </row>
     <row r="117" spans="1:6">
       <c r="B117" s="31" t="s">
+        <v>141</v>
+      </c>
+      <c r="C117" s="31" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6">
+      <c r="B118" s="31" t="s">
+        <v>143</v>
+      </c>
+      <c r="C118" s="31" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6">
+      <c r="B119" s="31" t="s">
         <v>145</v>
       </c>
-      <c r="C117" s="12"/>
-    </row>
-    <row r="120" spans="1:6" s="9" customFormat="1">
-      <c r="A120" s="9" t="s">
+      <c r="C119" s="12"/>
+    </row>
+    <row r="122" spans="1:6" s="9" customFormat="1">
+      <c r="A122" s="9" t="s">
         <v>146</v>
       </c>
-      <c r="B120" s="8"/>
-    </row>
-    <row r="121" spans="1:6">
-      <c r="A121" t="s">
+      <c r="B122" s="8"/>
+    </row>
+    <row r="123" spans="1:6">
+      <c r="A123" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="122" spans="1:6">
-      <c r="B122" s="39" t="s">
+    <row r="124" spans="1:6">
+      <c r="B124" s="39" t="s">
         <v>148</v>
-      </c>
-    </row>
-    <row r="123" spans="1:6">
-      <c r="B123" s="15" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="124" spans="1:6">
-      <c r="B124" s="30" t="s">
-        <v>150</v>
-      </c>
-      <c r="C124" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="125" spans="1:6">
       <c r="B125" s="15" t="s">
-        <v>137</v>
+        <v>149</v>
       </c>
     </row>
     <row r="126" spans="1:6">
       <c r="B126" s="30" t="s">
-        <v>151</v>
+        <v>150</v>
+      </c>
+      <c r="C126" t="s">
+        <v>150</v>
       </c>
     </row>
     <row r="127" spans="1:6">
       <c r="B127" s="15" t="s">
-        <v>152</v>
+        <v>137</v>
       </c>
     </row>
     <row r="128" spans="1:6">
       <c r="B128" s="30" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
     </row>
     <row r="129" spans="1:2">
       <c r="B129" s="15" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="130" spans="1:2">
+      <c r="B130" s="30" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="131" spans="1:2">
+      <c r="B131" s="15" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="130" spans="1:2">
-      <c r="B130" s="40" t="s">
+    <row r="132" spans="1:2">
+      <c r="B132" s="40" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="132" spans="1:2" ht="240" customHeight="1">
-      <c r="B132" s="34" t="s">
+    <row r="134" spans="1:2" ht="240" customHeight="1">
+      <c r="B134" s="34" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="136" spans="1:2">
-      <c r="A136" t="s">
+    <row r="138" spans="1:2">
+      <c r="A138" t="s">
         <v>157</v>
       </c>
-      <c r="B136" s="6" t="s">
+      <c r="B138" s="6" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="139" spans="1:2">
-      <c r="B139" s="6" t="s">
+    <row r="141" spans="1:2">
+      <c r="B141" s="6" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="140" spans="1:2">
-      <c r="B140" s="6" t="s">
+    <row r="142" spans="1:2">
+      <c r="B142" s="6" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="145" spans="2:3">
-      <c r="B145" s="42"/>
-      <c r="C145" s="41"/>
-    </row>
-    <row r="179" spans="1:3">
-      <c r="A179" t="s">
+    <row r="147" spans="2:3">
+      <c r="B147" s="42"/>
+      <c r="C147" s="41"/>
+    </row>
+    <row r="181" spans="1:3">
+      <c r="A181" t="s">
         <v>161</v>
       </c>
-      <c r="B179" s="6" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="180" spans="1:3">
-      <c r="B180" s="32" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="181" spans="1:3">
-      <c r="B181" s="31" t="s">
-        <v>162</v>
-      </c>
-      <c r="C181" t="s">
+      <c r="B181" s="6" t="s">
         <v>162</v>
       </c>
     </row>
     <row r="182" spans="1:3">
       <c r="B182" s="32" t="s">
-        <v>137</v>
+        <v>149</v>
       </c>
     </row>
     <row r="183" spans="1:3">
       <c r="B183" s="31" t="s">
-        <v>163</v>
+        <v>162</v>
+      </c>
+      <c r="C183" t="s">
+        <v>162</v>
       </c>
     </row>
     <row r="184" spans="1:3">
       <c r="B184" s="32" t="s">
-        <v>152</v>
+        <v>137</v>
       </c>
     </row>
     <row r="185" spans="1:3">
       <c r="B185" s="31" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="186" spans="1:3">
       <c r="B186" s="32" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="187" spans="1:3">
+      <c r="B187" s="31" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="188" spans="1:3">
+      <c r="B188" s="32" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="187" spans="1:3">
-      <c r="B187" s="33" t="s">
+    <row r="189" spans="1:3">
+      <c r="B189" s="33" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="189" spans="1:3" ht="240" customHeight="1">
-      <c r="B189" s="34" t="s">
+    <row r="191" spans="1:3" ht="240" customHeight="1">
+      <c r="B191" s="34" t="s">
         <v>166</v>
       </c>
     </row>
@@ -3753,48 +4473,48 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" s="56" customFormat="1" ht="30" customHeight="1">
-      <c r="A1" s="93" t="s">
+      <c r="A1" s="114" t="s">
         <v>473</v>
       </c>
-      <c r="B1" s="89"/>
-      <c r="C1" s="89"/>
-      <c r="D1" s="89"/>
-      <c r="E1" s="89"/>
-      <c r="F1" s="89"/>
-      <c r="G1" s="89"/>
-      <c r="H1" s="89"/>
-      <c r="I1" s="89"/>
-      <c r="J1" s="89"/>
-      <c r="K1" s="89"/>
-      <c r="L1" s="89"/>
-      <c r="M1" s="89"/>
+      <c r="B1" s="111"/>
+      <c r="C1" s="111"/>
+      <c r="D1" s="111"/>
+      <c r="E1" s="111"/>
+      <c r="F1" s="111"/>
+      <c r="G1" s="111"/>
+      <c r="H1" s="111"/>
+      <c r="I1" s="111"/>
+      <c r="J1" s="111"/>
+      <c r="K1" s="111"/>
+      <c r="L1" s="111"/>
+      <c r="M1" s="111"/>
       <c r="N1" s="55"/>
     </row>
     <row r="2" spans="1:20" s="56" customFormat="1" ht="15.95" customHeight="1">
-      <c r="A2" s="92" t="s">
+      <c r="A2" s="113" t="s">
         <v>474</v>
       </c>
-      <c r="B2" s="87"/>
-      <c r="D2" s="85" t="s">
+      <c r="B2" s="110"/>
+      <c r="D2" s="108" t="s">
         <v>475</v>
       </c>
-      <c r="E2" s="86"/>
-      <c r="F2" s="86"/>
-      <c r="G2" s="86"/>
-      <c r="H2" s="86"/>
-      <c r="I2" s="86"/>
-      <c r="J2" s="86"/>
-      <c r="K2" s="86"/>
-      <c r="L2" s="87"/>
+      <c r="E2" s="109"/>
+      <c r="F2" s="109"/>
+      <c r="G2" s="109"/>
+      <c r="H2" s="109"/>
+      <c r="I2" s="109"/>
+      <c r="J2" s="109"/>
+      <c r="K2" s="109"/>
+      <c r="L2" s="110"/>
       <c r="N2" s="55"/>
-      <c r="O2" s="94" t="s">
+      <c r="O2" s="106" t="s">
         <v>3</v>
       </c>
-      <c r="P2" s="95"/>
-      <c r="Q2" s="95"/>
-      <c r="R2" s="95"/>
-      <c r="S2" s="95"/>
-      <c r="T2" s="95"/>
+      <c r="P2" s="107"/>
+      <c r="Q2" s="107"/>
+      <c r="R2" s="107"/>
+      <c r="S2" s="107"/>
+      <c r="T2" s="107"/>
     </row>
     <row r="3" spans="1:20" s="56" customFormat="1" ht="36" customHeight="1">
       <c r="A3" s="62" t="s">
@@ -4332,21 +5052,21 @@
       <c r="G12" s="75"/>
     </row>
     <row r="13" spans="1:20">
-      <c r="A13" s="88" t="s">
+      <c r="A13" s="102" t="s">
         <v>534</v>
       </c>
-      <c r="B13" s="90"/>
-      <c r="C13" s="90"/>
-      <c r="D13" s="90"/>
-      <c r="E13" s="90"/>
-      <c r="F13" s="90"/>
-      <c r="G13" s="90"/>
-      <c r="H13" s="90"/>
-      <c r="I13" s="90"/>
-      <c r="J13" s="90"/>
-      <c r="K13" s="90"/>
-      <c r="L13" s="90"/>
-      <c r="M13" s="90"/>
+      <c r="B13" s="100"/>
+      <c r="C13" s="100"/>
+      <c r="D13" s="100"/>
+      <c r="E13" s="100"/>
+      <c r="F13" s="100"/>
+      <c r="G13" s="100"/>
+      <c r="H13" s="100"/>
+      <c r="I13" s="100"/>
+      <c r="J13" s="100"/>
+      <c r="K13" s="100"/>
+      <c r="L13" s="100"/>
+      <c r="M13" s="100"/>
     </row>
     <row r="14" spans="1:20">
       <c r="E14" s="74"/>
@@ -4399,48 +5119,48 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" s="56" customFormat="1" ht="30" customHeight="1">
-      <c r="A1" s="93" t="s">
+      <c r="A1" s="114" t="s">
         <v>535</v>
       </c>
-      <c r="B1" s="89"/>
-      <c r="C1" s="89"/>
-      <c r="D1" s="89"/>
-      <c r="E1" s="89"/>
-      <c r="F1" s="89"/>
-      <c r="G1" s="89"/>
-      <c r="H1" s="89"/>
-      <c r="I1" s="89"/>
-      <c r="J1" s="89"/>
-      <c r="K1" s="89"/>
-      <c r="L1" s="89"/>
-      <c r="M1" s="89"/>
+      <c r="B1" s="111"/>
+      <c r="C1" s="111"/>
+      <c r="D1" s="111"/>
+      <c r="E1" s="111"/>
+      <c r="F1" s="111"/>
+      <c r="G1" s="111"/>
+      <c r="H1" s="111"/>
+      <c r="I1" s="111"/>
+      <c r="J1" s="111"/>
+      <c r="K1" s="111"/>
+      <c r="L1" s="111"/>
+      <c r="M1" s="111"/>
       <c r="N1" s="55"/>
     </row>
     <row r="2" spans="1:20" s="56" customFormat="1" ht="15.95" customHeight="1">
-      <c r="A2" s="92" t="s">
+      <c r="A2" s="113" t="s">
         <v>474</v>
       </c>
-      <c r="B2" s="87"/>
-      <c r="D2" s="85" t="s">
+      <c r="B2" s="110"/>
+      <c r="D2" s="108" t="s">
         <v>475</v>
       </c>
-      <c r="E2" s="86"/>
-      <c r="F2" s="86"/>
-      <c r="G2" s="86"/>
-      <c r="H2" s="86"/>
-      <c r="I2" s="86"/>
-      <c r="J2" s="86"/>
-      <c r="K2" s="86"/>
-      <c r="L2" s="87"/>
+      <c r="E2" s="109"/>
+      <c r="F2" s="109"/>
+      <c r="G2" s="109"/>
+      <c r="H2" s="109"/>
+      <c r="I2" s="109"/>
+      <c r="J2" s="109"/>
+      <c r="K2" s="109"/>
+      <c r="L2" s="110"/>
       <c r="N2" s="55"/>
-      <c r="O2" s="94" t="s">
+      <c r="O2" s="106" t="s">
         <v>3</v>
       </c>
-      <c r="P2" s="95"/>
-      <c r="Q2" s="95"/>
-      <c r="R2" s="95"/>
-      <c r="S2" s="95"/>
-      <c r="T2" s="95"/>
+      <c r="P2" s="107"/>
+      <c r="Q2" s="107"/>
+      <c r="R2" s="107"/>
+      <c r="S2" s="107"/>
+      <c r="T2" s="107"/>
     </row>
     <row r="3" spans="1:20" s="56" customFormat="1" ht="36" customHeight="1">
       <c r="A3" s="62" t="s">
@@ -4968,21 +5688,21 @@
       <c r="G12" s="75"/>
     </row>
     <row r="13" spans="1:20">
-      <c r="A13" s="88" t="s">
+      <c r="A13" s="102" t="s">
         <v>560</v>
       </c>
-      <c r="B13" s="90"/>
-      <c r="C13" s="90"/>
-      <c r="D13" s="90"/>
-      <c r="E13" s="90"/>
-      <c r="F13" s="90"/>
-      <c r="G13" s="90"/>
-      <c r="H13" s="90"/>
-      <c r="I13" s="90"/>
-      <c r="J13" s="90"/>
-      <c r="K13" s="90"/>
-      <c r="L13" s="90"/>
-      <c r="M13" s="90"/>
+      <c r="B13" s="100"/>
+      <c r="C13" s="100"/>
+      <c r="D13" s="100"/>
+      <c r="E13" s="100"/>
+      <c r="F13" s="100"/>
+      <c r="G13" s="100"/>
+      <c r="H13" s="100"/>
+      <c r="I13" s="100"/>
+      <c r="J13" s="100"/>
+      <c r="K13" s="100"/>
+      <c r="L13" s="100"/>
+      <c r="M13" s="100"/>
     </row>
     <row r="14" spans="1:20">
       <c r="E14" s="74"/>
@@ -5035,48 +5755,48 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" s="56" customFormat="1" ht="30" customHeight="1">
-      <c r="A1" s="93" t="s">
+      <c r="A1" s="114" t="s">
         <v>561</v>
       </c>
-      <c r="B1" s="89"/>
-      <c r="C1" s="89"/>
-      <c r="D1" s="89"/>
-      <c r="E1" s="89"/>
-      <c r="F1" s="89"/>
-      <c r="G1" s="89"/>
-      <c r="H1" s="89"/>
-      <c r="I1" s="89"/>
-      <c r="J1" s="89"/>
-      <c r="K1" s="89"/>
-      <c r="L1" s="89"/>
-      <c r="M1" s="89"/>
+      <c r="B1" s="111"/>
+      <c r="C1" s="111"/>
+      <c r="D1" s="111"/>
+      <c r="E1" s="111"/>
+      <c r="F1" s="111"/>
+      <c r="G1" s="111"/>
+      <c r="H1" s="111"/>
+      <c r="I1" s="111"/>
+      <c r="J1" s="111"/>
+      <c r="K1" s="111"/>
+      <c r="L1" s="111"/>
+      <c r="M1" s="111"/>
       <c r="N1" s="55"/>
     </row>
     <row r="2" spans="1:20" s="56" customFormat="1" ht="15.95" customHeight="1">
-      <c r="A2" s="92" t="s">
+      <c r="A2" s="113" t="s">
         <v>474</v>
       </c>
-      <c r="B2" s="87"/>
-      <c r="D2" s="85" t="s">
+      <c r="B2" s="110"/>
+      <c r="D2" s="108" t="s">
         <v>475</v>
       </c>
-      <c r="E2" s="86"/>
-      <c r="F2" s="86"/>
-      <c r="G2" s="86"/>
-      <c r="H2" s="86"/>
-      <c r="I2" s="86"/>
-      <c r="J2" s="86"/>
-      <c r="K2" s="86"/>
-      <c r="L2" s="87"/>
+      <c r="E2" s="109"/>
+      <c r="F2" s="109"/>
+      <c r="G2" s="109"/>
+      <c r="H2" s="109"/>
+      <c r="I2" s="109"/>
+      <c r="J2" s="109"/>
+      <c r="K2" s="109"/>
+      <c r="L2" s="110"/>
       <c r="N2" s="55"/>
-      <c r="O2" s="94" t="s">
+      <c r="O2" s="106" t="s">
         <v>3</v>
       </c>
-      <c r="P2" s="95"/>
-      <c r="Q2" s="95"/>
-      <c r="R2" s="95"/>
-      <c r="S2" s="95"/>
-      <c r="T2" s="95"/>
+      <c r="P2" s="107"/>
+      <c r="Q2" s="107"/>
+      <c r="R2" s="107"/>
+      <c r="S2" s="107"/>
+      <c r="T2" s="107"/>
     </row>
     <row r="3" spans="1:20" s="56" customFormat="1" ht="36" customHeight="1">
       <c r="A3" s="62" t="s">
@@ -5604,21 +6324,21 @@
       <c r="G12" s="75"/>
     </row>
     <row r="13" spans="1:20">
-      <c r="A13" s="88" t="s">
+      <c r="A13" s="102" t="s">
         <v>41</v>
       </c>
-      <c r="B13" s="90"/>
-      <c r="C13" s="90"/>
-      <c r="D13" s="90"/>
-      <c r="E13" s="90"/>
-      <c r="F13" s="90"/>
-      <c r="G13" s="90"/>
-      <c r="H13" s="90"/>
-      <c r="I13" s="90"/>
-      <c r="J13" s="90"/>
-      <c r="K13" s="90"/>
-      <c r="L13" s="90"/>
-      <c r="M13" s="90"/>
+      <c r="B13" s="100"/>
+      <c r="C13" s="100"/>
+      <c r="D13" s="100"/>
+      <c r="E13" s="100"/>
+      <c r="F13" s="100"/>
+      <c r="G13" s="100"/>
+      <c r="H13" s="100"/>
+      <c r="I13" s="100"/>
+      <c r="J13" s="100"/>
+      <c r="K13" s="100"/>
+      <c r="L13" s="100"/>
+      <c r="M13" s="100"/>
     </row>
     <row r="14" spans="1:20">
       <c r="E14" s="74"/>
@@ -5671,48 +6391,48 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" s="56" customFormat="1" ht="30" customHeight="1">
-      <c r="A1" s="93" t="s">
+      <c r="A1" s="114" t="s">
         <v>561</v>
       </c>
-      <c r="B1" s="89"/>
-      <c r="C1" s="89"/>
-      <c r="D1" s="89"/>
-      <c r="E1" s="89"/>
-      <c r="F1" s="89"/>
-      <c r="G1" s="89"/>
-      <c r="H1" s="89"/>
-      <c r="I1" s="89"/>
-      <c r="J1" s="89"/>
-      <c r="K1" s="89"/>
-      <c r="L1" s="89"/>
-      <c r="M1" s="89"/>
+      <c r="B1" s="111"/>
+      <c r="C1" s="111"/>
+      <c r="D1" s="111"/>
+      <c r="E1" s="111"/>
+      <c r="F1" s="111"/>
+      <c r="G1" s="111"/>
+      <c r="H1" s="111"/>
+      <c r="I1" s="111"/>
+      <c r="J1" s="111"/>
+      <c r="K1" s="111"/>
+      <c r="L1" s="111"/>
+      <c r="M1" s="111"/>
       <c r="N1" s="55"/>
     </row>
     <row r="2" spans="1:20" s="56" customFormat="1" ht="15.95" customHeight="1">
-      <c r="A2" s="92" t="s">
+      <c r="A2" s="113" t="s">
         <v>474</v>
       </c>
-      <c r="B2" s="87"/>
-      <c r="D2" s="85" t="s">
+      <c r="B2" s="110"/>
+      <c r="D2" s="108" t="s">
         <v>475</v>
       </c>
-      <c r="E2" s="86"/>
-      <c r="F2" s="86"/>
-      <c r="G2" s="86"/>
-      <c r="H2" s="86"/>
-      <c r="I2" s="86"/>
-      <c r="J2" s="86"/>
-      <c r="K2" s="86"/>
-      <c r="L2" s="87"/>
+      <c r="E2" s="109"/>
+      <c r="F2" s="109"/>
+      <c r="G2" s="109"/>
+      <c r="H2" s="109"/>
+      <c r="I2" s="109"/>
+      <c r="J2" s="109"/>
+      <c r="K2" s="109"/>
+      <c r="L2" s="110"/>
       <c r="N2" s="55"/>
-      <c r="O2" s="94" t="s">
+      <c r="O2" s="106" t="s">
         <v>3</v>
       </c>
-      <c r="P2" s="95"/>
-      <c r="Q2" s="95"/>
-      <c r="R2" s="95"/>
-      <c r="S2" s="95"/>
-      <c r="T2" s="95"/>
+      <c r="P2" s="107"/>
+      <c r="Q2" s="107"/>
+      <c r="R2" s="107"/>
+      <c r="S2" s="107"/>
+      <c r="T2" s="107"/>
     </row>
     <row r="3" spans="1:20" s="56" customFormat="1" ht="36" customHeight="1">
       <c r="A3" s="62" t="s">
@@ -6256,21 +6976,21 @@
       <c r="G12" s="75"/>
     </row>
     <row r="13" spans="1:20">
-      <c r="A13" s="88" t="s">
+      <c r="A13" s="102" t="s">
         <v>41</v>
       </c>
-      <c r="B13" s="90"/>
-      <c r="C13" s="90"/>
-      <c r="D13" s="90"/>
-      <c r="E13" s="90"/>
-      <c r="F13" s="90"/>
-      <c r="G13" s="90"/>
-      <c r="H13" s="90"/>
-      <c r="I13" s="90"/>
-      <c r="J13" s="90"/>
-      <c r="K13" s="90"/>
-      <c r="L13" s="90"/>
-      <c r="M13" s="90"/>
+      <c r="B13" s="100"/>
+      <c r="C13" s="100"/>
+      <c r="D13" s="100"/>
+      <c r="E13" s="100"/>
+      <c r="F13" s="100"/>
+      <c r="G13" s="100"/>
+      <c r="H13" s="100"/>
+      <c r="I13" s="100"/>
+      <c r="J13" s="100"/>
+      <c r="K13" s="100"/>
+      <c r="L13" s="100"/>
+      <c r="M13" s="100"/>
     </row>
     <row r="14" spans="1:20">
       <c r="E14" s="74"/>
@@ -6322,47 +7042,47 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="30" customHeight="1">
-      <c r="A1" s="93" t="s">
+      <c r="A1" s="114" t="s">
         <v>602</v>
       </c>
-      <c r="B1" s="89"/>
-      <c r="C1" s="90"/>
-      <c r="D1" s="91"/>
-      <c r="E1" s="90"/>
-      <c r="F1" s="90"/>
-      <c r="G1" s="90"/>
-      <c r="H1" s="90"/>
-      <c r="I1" s="90"/>
-      <c r="J1" s="90"/>
-      <c r="K1" s="90"/>
-      <c r="L1" s="90"/>
-      <c r="M1" s="90"/>
+      <c r="B1" s="111"/>
+      <c r="C1" s="100"/>
+      <c r="D1" s="112"/>
+      <c r="E1" s="100"/>
+      <c r="F1" s="100"/>
+      <c r="G1" s="100"/>
+      <c r="H1" s="100"/>
+      <c r="I1" s="100"/>
+      <c r="J1" s="100"/>
+      <c r="K1" s="100"/>
+      <c r="L1" s="100"/>
+      <c r="M1" s="100"/>
     </row>
     <row r="2" spans="1:20" ht="15.95" customHeight="1">
-      <c r="A2" s="92" t="s">
+      <c r="A2" s="113" t="s">
         <v>603</v>
       </c>
-      <c r="B2" s="87"/>
+      <c r="B2" s="110"/>
       <c r="C2" s="56"/>
-      <c r="D2" s="85" t="s">
+      <c r="D2" s="108" t="s">
         <v>475</v>
       </c>
-      <c r="E2" s="86"/>
-      <c r="F2" s="86"/>
-      <c r="G2" s="86"/>
-      <c r="H2" s="86"/>
-      <c r="I2" s="86"/>
-      <c r="J2" s="86"/>
-      <c r="K2" s="86"/>
-      <c r="L2" s="87"/>
-      <c r="O2" s="94" t="s">
+      <c r="E2" s="109"/>
+      <c r="F2" s="109"/>
+      <c r="G2" s="109"/>
+      <c r="H2" s="109"/>
+      <c r="I2" s="109"/>
+      <c r="J2" s="109"/>
+      <c r="K2" s="109"/>
+      <c r="L2" s="110"/>
+      <c r="O2" s="106" t="s">
         <v>3</v>
       </c>
-      <c r="P2" s="95"/>
-      <c r="Q2" s="95"/>
-      <c r="R2" s="95"/>
-      <c r="S2" s="95"/>
-      <c r="T2" s="95"/>
+      <c r="P2" s="107"/>
+      <c r="Q2" s="107"/>
+      <c r="R2" s="107"/>
+      <c r="S2" s="107"/>
+      <c r="T2" s="107"/>
     </row>
     <row r="3" spans="1:20" ht="36" customHeight="1">
       <c r="A3" s="62" t="s">
@@ -6894,19 +7614,19 @@
       <c r="L12" s="75"/>
     </row>
     <row r="13" spans="1:20" ht="12.95" customHeight="1">
-      <c r="A13" s="88"/>
-      <c r="B13" s="89"/>
-      <c r="C13" s="90"/>
-      <c r="D13" s="91"/>
-      <c r="E13" s="90"/>
-      <c r="F13" s="90"/>
-      <c r="G13" s="90"/>
-      <c r="H13" s="90"/>
-      <c r="I13" s="90"/>
-      <c r="J13" s="90"/>
-      <c r="K13" s="90"/>
-      <c r="L13" s="90"/>
-      <c r="M13" s="90"/>
+      <c r="A13" s="102"/>
+      <c r="B13" s="111"/>
+      <c r="C13" s="100"/>
+      <c r="D13" s="112"/>
+      <c r="E13" s="100"/>
+      <c r="F13" s="100"/>
+      <c r="G13" s="100"/>
+      <c r="H13" s="100"/>
+      <c r="I13" s="100"/>
+      <c r="J13" s="100"/>
+      <c r="K13" s="100"/>
+      <c r="L13" s="100"/>
+      <c r="M13" s="100"/>
     </row>
     <row r="14" spans="1:20" ht="29.25" customHeight="1">
       <c r="A14" s="75" t="s">
@@ -6958,545 +7678,656 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="B2:K125"/>
+  <dimension ref="A2:K138"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="9.140625" style="12" customWidth="1"/>
+    <col min="1" max="1" width="19.5703125" style="12" customWidth="1"/>
     <col min="2" max="2" width="137.85546875" style="12" customWidth="1"/>
-    <col min="3" max="5" width="9.140625" style="12" customWidth="1"/>
+    <col min="3" max="3" width="36.85546875" style="12" customWidth="1"/>
+    <col min="4" max="5" width="9.140625" style="12" customWidth="1"/>
     <col min="6" max="16384" width="9.140625" style="12"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:3">
-      <c r="B2" s="1" t="s">
+    <row r="2" spans="1:3" ht="20.25">
+      <c r="A2" s="95" t="s">
+        <v>638</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" s="96" t="s">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="15.75" thickBot="1">
+      <c r="A4" s="91" t="s">
+        <v>640</v>
+      </c>
+      <c r="B4" s="91" t="s">
+        <v>641</v>
+      </c>
+      <c r="C4" s="91" t="s">
+        <v>642</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="97.5">
+      <c r="A5" s="92" t="s">
+        <v>643</v>
+      </c>
+      <c r="B5" s="93" t="s">
+        <v>653</v>
+      </c>
+      <c r="C5" s="93" t="s">
+        <v>652</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="42.75">
+      <c r="A6" s="92" t="s">
+        <v>644</v>
+      </c>
+      <c r="B6" s="93" t="s">
+        <v>655</v>
+      </c>
+      <c r="C6" s="93" t="s">
+        <v>654</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="119.25">
+      <c r="A7" s="92" t="s">
+        <v>645</v>
+      </c>
+      <c r="B7" s="93" t="s">
+        <v>657</v>
+      </c>
+      <c r="C7" s="93" t="s">
+        <v>656</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="239.25">
+      <c r="A8" s="92" t="s">
+        <v>646</v>
+      </c>
+      <c r="B8" s="93" t="s">
+        <v>659</v>
+      </c>
+      <c r="C8" s="93" t="s">
+        <v>658</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="87.75">
+      <c r="A9" s="92" t="s">
+        <v>647</v>
+      </c>
+      <c r="B9" s="93" t="s">
+        <v>661</v>
+      </c>
+      <c r="C9" s="93" t="s">
+        <v>660</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="65.25">
+      <c r="A10" s="92" t="s">
+        <v>648</v>
+      </c>
+      <c r="B10" s="93" t="s">
+        <v>663</v>
+      </c>
+      <c r="C10" s="94" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="130.5">
+      <c r="A11" s="92" t="s">
+        <v>649</v>
+      </c>
+      <c r="B11" s="94" t="s">
+        <v>665</v>
+      </c>
+      <c r="C11" s="93" t="s">
+        <v>664</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="21.75">
+      <c r="A12" s="92" t="s">
+        <v>650</v>
+      </c>
+      <c r="B12" s="93" t="s">
+        <v>666</v>
+      </c>
+      <c r="C12" s="94" t="s">
+        <v>651</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" s="53" customFormat="1"/>
+    <row r="15" spans="1:3">
+      <c r="B15" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="C15" s="12" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="3" spans="2:3">
-      <c r="C3" s="12" t="s">
+    <row r="16" spans="1:3">
+      <c r="C16" s="12" t="s">
         <v>169</v>
-      </c>
-    </row>
-    <row r="4" spans="2:3">
-      <c r="B4" s="1" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="6" spans="2:3">
-      <c r="B6" s="1" t="s">
-        <v>171</v>
-      </c>
-      <c r="C6" s="12" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="7" spans="2:3">
-      <c r="B7" t="s">
-        <v>173</v>
-      </c>
-      <c r="C7" s="12" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="9" spans="2:3">
-      <c r="B9" s="1" t="s">
-        <v>175</v>
-      </c>
-      <c r="C9" s="12" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="10" spans="2:3">
-      <c r="B10" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="12" spans="2:3">
-      <c r="B12" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="C12" s="12" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="13" spans="2:3">
-      <c r="B13" t="s">
-        <v>180</v>
-      </c>
-      <c r="C13" s="12" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="15" spans="2:3">
-      <c r="B15" s="1" t="s">
-        <v>182</v>
       </c>
     </row>
     <row r="17" spans="2:11">
       <c r="B17" s="1" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="19" spans="2:11">
+      <c r="B19" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="C19" s="12" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="20" spans="2:11">
+      <c r="B20" t="s">
+        <v>173</v>
+      </c>
+      <c r="C20" s="12" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="22" spans="2:11">
+      <c r="B22" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="C22" s="12" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="23" spans="2:11">
+      <c r="B23" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="25" spans="2:11">
+      <c r="B25" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="C25" s="12" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="26" spans="2:11">
+      <c r="B26" t="s">
+        <v>180</v>
+      </c>
+      <c r="C26" s="12" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="28" spans="2:11">
+      <c r="B28" s="1" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="30" spans="2:11">
+      <c r="B30" s="1" t="s">
         <v>183</v>
       </c>
-      <c r="C17" s="12" t="s">
+      <c r="C30" s="12" t="s">
         <v>184</v>
-      </c>
-    </row>
-    <row r="19" spans="2:11">
-      <c r="B19" s="12" t="s">
-        <v>185</v>
-      </c>
-      <c r="C19" s="12" t="s">
-        <v>185</v>
-      </c>
-      <c r="K19" s="12" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="20" spans="2:11">
-      <c r="B20" s="12" t="s">
-        <v>187</v>
-      </c>
-      <c r="C20" s="12" t="s">
-        <v>187</v>
-      </c>
-      <c r="K20" s="12" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="22" spans="2:11">
-      <c r="B22" s="12" t="s">
-        <v>189</v>
-      </c>
-      <c r="C22" s="12" t="s">
-        <v>189</v>
-      </c>
-      <c r="K22" s="12" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="24" spans="2:11">
-      <c r="B24" s="12" t="s">
-        <v>191</v>
-      </c>
-      <c r="C24" s="12" t="s">
-        <v>191</v>
-      </c>
-      <c r="K24" s="12" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="25" spans="2:11">
-      <c r="B25" s="12" t="s">
-        <v>193</v>
-      </c>
-      <c r="C25" s="12" t="s">
-        <v>193</v>
-      </c>
-      <c r="K25" s="12" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="28" spans="2:11" s="53" customFormat="1">
-      <c r="B28" s="53" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="29" spans="2:11">
-      <c r="B29" s="12" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="31" spans="2:11">
-      <c r="B31" s="12" t="s">
-        <v>196</v>
-      </c>
-      <c r="C31" s="12" t="s">
-        <v>197</v>
       </c>
     </row>
     <row r="32" spans="2:11">
       <c r="B32" s="12" t="s">
+        <v>185</v>
+      </c>
+      <c r="C32" s="12" t="s">
+        <v>185</v>
+      </c>
+      <c r="K32" s="12" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="33" spans="2:11">
+      <c r="B33" s="12" t="s">
+        <v>187</v>
+      </c>
+      <c r="C33" s="12" t="s">
+        <v>187</v>
+      </c>
+      <c r="K33" s="12" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="35" spans="2:11">
+      <c r="B35" s="12" t="s">
+        <v>189</v>
+      </c>
+      <c r="C35" s="12" t="s">
+        <v>189</v>
+      </c>
+      <c r="K35" s="12" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="37" spans="2:11">
+      <c r="B37" s="12" t="s">
+        <v>191</v>
+      </c>
+      <c r="C37" s="12" t="s">
+        <v>191</v>
+      </c>
+      <c r="K37" s="12" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="38" spans="2:11">
+      <c r="B38" s="12" t="s">
+        <v>193</v>
+      </c>
+      <c r="C38" s="12" t="s">
+        <v>193</v>
+      </c>
+      <c r="K38" s="12" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="41" spans="2:11" s="53" customFormat="1">
+      <c r="B41" s="53" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="42" spans="2:11">
+      <c r="B42" s="12" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="44" spans="2:11">
+      <c r="B44" s="12" t="s">
+        <v>196</v>
+      </c>
+      <c r="C44" s="12" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="45" spans="2:11">
+      <c r="B45" s="12" t="s">
         <v>198</v>
       </c>
-      <c r="C32" s="12" t="s">
+      <c r="C45" s="12" t="s">
         <v>199</v>
       </c>
     </row>
-    <row r="34" spans="2:6">
-      <c r="B34" s="12" t="s">
+    <row r="47" spans="2:11">
+      <c r="B47" s="12" t="s">
         <v>200</v>
-      </c>
-    </row>
-    <row r="36" spans="2:6">
-      <c r="B36" s="12" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="37" spans="2:6">
-      <c r="B37" s="12" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="39" spans="2:6">
-      <c r="B39" s="12" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="41" spans="2:6">
-      <c r="B41" s="12" t="s">
-        <v>204</v>
-      </c>
-      <c r="C41" s="78" t="s">
-        <v>205</v>
-      </c>
-      <c r="D41" s="12" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="42" spans="2:6" s="81" customFormat="1"/>
-    <row r="43" spans="2:6" s="53" customFormat="1">
-      <c r="B43" s="53" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="45" spans="2:6">
-      <c r="B45" s="12" t="s">
-        <v>208</v>
-      </c>
-      <c r="D45" s="12" t="s">
-        <v>209</v>
-      </c>
-      <c r="F45" s="12" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="47" spans="2:6">
-      <c r="B47" s="12" t="s">
-        <v>211</v>
-      </c>
-      <c r="F47" s="12" t="s">
-        <v>212</v>
       </c>
     </row>
     <row r="49" spans="2:6">
       <c r="B49" s="12" t="s">
-        <v>213</v>
-      </c>
-      <c r="F49" s="12" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="51" spans="2:6">
-      <c r="B51" s="12" t="s">
-        <v>43</v>
+        <v>201</v>
+      </c>
+    </row>
+    <row r="50" spans="2:6">
+      <c r="B50" s="12" t="s">
+        <v>202</v>
       </c>
     </row>
     <row r="52" spans="2:6">
       <c r="B52" s="12" t="s">
-        <v>215</v>
+        <v>203</v>
       </c>
     </row>
     <row r="54" spans="2:6">
       <c r="B54" s="12" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="55" spans="2:6">
-      <c r="B55" s="12" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="56" spans="2:6">
-      <c r="B56" s="12" t="s">
-        <v>218</v>
+        <v>204</v>
+      </c>
+      <c r="C54" s="78" t="s">
+        <v>205</v>
+      </c>
+      <c r="D54" s="12" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="55" spans="2:6" s="81" customFormat="1"/>
+    <row r="56" spans="2:6" s="53" customFormat="1">
+      <c r="B56" s="53" t="s">
+        <v>207</v>
       </c>
     </row>
     <row r="58" spans="2:6">
       <c r="B58" s="12" t="s">
+        <v>208</v>
+      </c>
+      <c r="D58" s="12" t="s">
+        <v>209</v>
+      </c>
+      <c r="F58" s="12" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="60" spans="2:6">
+      <c r="B60" s="12" t="s">
+        <v>211</v>
+      </c>
+      <c r="F60" s="12" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="62" spans="2:6">
+      <c r="B62" s="12" t="s">
+        <v>213</v>
+      </c>
+      <c r="F62" s="12" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="64" spans="2:6">
+      <c r="B64" s="12" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="65" spans="2:3">
+      <c r="B65" s="12" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="67" spans="2:3">
+      <c r="B67" s="12" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="68" spans="2:3">
+      <c r="B68" s="12" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="69" spans="2:3">
+      <c r="B69" s="12" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="71" spans="2:3">
+      <c r="B71" s="12" t="s">
         <v>219</v>
       </c>
     </row>
-    <row r="61" spans="2:6">
-      <c r="B61" s="51" t="s">
+    <row r="74" spans="2:3">
+      <c r="B74" s="51" t="s">
         <v>220</v>
       </c>
-      <c r="C61" s="51" t="s">
+      <c r="C74" s="51" t="s">
         <v>221</v>
       </c>
     </row>
-    <row r="62" spans="2:6">
-      <c r="B62" s="25" t="s">
+    <row r="75" spans="2:3">
+      <c r="B75" s="25" t="s">
         <v>222</v>
       </c>
-      <c r="C62" s="52" t="s">
+      <c r="C75" s="52" t="s">
         <v>223</v>
       </c>
     </row>
-    <row r="63" spans="2:6">
-      <c r="B63" s="25" t="s">
+    <row r="76" spans="2:3">
+      <c r="B76" s="25" t="s">
         <v>224</v>
       </c>
-      <c r="C63" s="52" t="s">
+      <c r="C76" s="52" t="s">
         <v>225</v>
       </c>
     </row>
-    <row r="64" spans="2:6">
-      <c r="B64" s="25" t="s">
+    <row r="77" spans="2:3">
+      <c r="B77" s="25" t="s">
         <v>226</v>
       </c>
-      <c r="C64" s="52" t="s">
+      <c r="C77" s="52" t="s">
         <v>227</v>
       </c>
     </row>
-    <row r="65" spans="2:4">
-      <c r="B65" s="25" t="s">
+    <row r="78" spans="2:3">
+      <c r="B78" s="25" t="s">
         <v>228</v>
       </c>
-      <c r="C65" s="52" t="s">
+      <c r="C78" s="52" t="s">
         <v>229</v>
       </c>
     </row>
-    <row r="66" spans="2:4">
-      <c r="B66" s="25" t="s">
+    <row r="79" spans="2:3">
+      <c r="B79" s="25" t="s">
         <v>230</v>
       </c>
-      <c r="C66" s="52" t="s">
+      <c r="C79" s="52" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="67" spans="2:4">
-      <c r="B67" s="25" t="s">
+    <row r="80" spans="2:3">
+      <c r="B80" s="25" t="s">
         <v>232</v>
       </c>
-      <c r="C67" s="52" t="s">
+      <c r="C80" s="52" t="s">
         <v>233</v>
       </c>
     </row>
-    <row r="72" spans="2:4" ht="18" customHeight="1">
-      <c r="B72" s="48" t="s">
+    <row r="85" spans="2:4" ht="18" customHeight="1">
+      <c r="B85" s="48" t="s">
         <v>234</v>
       </c>
     </row>
-    <row r="73" spans="2:4">
-      <c r="B73" s="13" t="s">
+    <row r="86" spans="2:4">
+      <c r="B86" s="13" t="s">
         <v>235</v>
       </c>
     </row>
-    <row r="74" spans="2:4">
-      <c r="B74" s="49" t="s">
+    <row r="87" spans="2:4">
+      <c r="B87" s="49" t="s">
         <v>236</v>
       </c>
     </row>
-    <row r="76" spans="2:4" ht="18" customHeight="1">
-      <c r="B76" s="48" t="s">
+    <row r="89" spans="2:4" ht="18" customHeight="1">
+      <c r="B89" s="48" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="77" spans="2:4">
-      <c r="B77" s="50" t="s">
+    <row r="90" spans="2:4">
+      <c r="B90" s="50" t="s">
         <v>238</v>
       </c>
     </row>
-    <row r="78" spans="2:4">
-      <c r="B78" s="50" t="s">
+    <row r="91" spans="2:4">
+      <c r="B91" s="50" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="79" spans="2:4">
-      <c r="B79" s="50" t="s">
+    <row r="92" spans="2:4">
+      <c r="B92" s="50" t="s">
         <v>240</v>
       </c>
     </row>
-    <row r="80" spans="2:4">
-      <c r="D80" s="31"/>
-    </row>
-    <row r="81" spans="2:4" ht="18" customHeight="1">
-      <c r="B81" s="48" t="s">
+    <row r="93" spans="2:4">
+      <c r="D93" s="31"/>
+    </row>
+    <row r="94" spans="2:4" ht="18" customHeight="1">
+      <c r="B94" s="48" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="82" spans="2:4">
-      <c r="B82" s="50" t="s">
+    <row r="95" spans="2:4">
+      <c r="B95" s="50" t="s">
         <v>242</v>
       </c>
-      <c r="D82" s="31"/>
-    </row>
-    <row r="83" spans="2:4">
-      <c r="B83" s="50" t="s">
+      <c r="D95" s="31"/>
+    </row>
+    <row r="96" spans="2:4">
+      <c r="B96" s="50" t="s">
         <v>243</v>
       </c>
-      <c r="D83" s="31"/>
-    </row>
-    <row r="84" spans="2:4">
-      <c r="B84" s="50" t="s">
+      <c r="D96" s="31"/>
+    </row>
+    <row r="97" spans="2:4">
+      <c r="B97" s="50" t="s">
         <v>244</v>
       </c>
-      <c r="D84" s="31"/>
-    </row>
-    <row r="86" spans="2:4" ht="18" customHeight="1">
-      <c r="B86" s="48" t="s">
+      <c r="D97" s="31"/>
+    </row>
+    <row r="99" spans="2:4" ht="18" customHeight="1">
+      <c r="B99" s="48" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="87" spans="2:4">
-      <c r="B87" s="13" t="s">
+    <row r="100" spans="2:4">
+      <c r="B100" s="13" t="s">
         <v>246</v>
       </c>
     </row>
-    <row r="88" spans="2:4">
-      <c r="B88" s="12" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="89" spans="2:4">
-      <c r="B89" s="14" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="90" spans="2:4">
-      <c r="B90" s="49" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="92" spans="2:4" ht="18" customHeight="1">
-      <c r="B92" s="48" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="93" spans="2:4">
-      <c r="B93" s="13" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="94" spans="2:4">
-      <c r="B94" s="49" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="95" spans="2:4">
-      <c r="B95" s="12" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="96" spans="2:4">
-      <c r="B96" s="14" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="97" spans="2:2">
-      <c r="B97" s="49" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="99" spans="2:2" ht="18" customHeight="1">
-      <c r="B99" s="48" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="100" spans="2:2">
-      <c r="B100" s="13" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="101" spans="2:2">
+    <row r="101" spans="2:4">
       <c r="B101" s="12" t="s">
         <v>247</v>
       </c>
     </row>
-    <row r="102" spans="2:2">
+    <row r="102" spans="2:4">
       <c r="B102" s="14" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="103" spans="2:4">
+      <c r="B103" s="49" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="105" spans="2:4" ht="18" customHeight="1">
+      <c r="B105" s="48" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="106" spans="2:4">
+      <c r="B106" s="13" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="107" spans="2:4">
+      <c r="B107" s="49" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="108" spans="2:4">
+      <c r="B108" s="12" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="109" spans="2:4">
+      <c r="B109" s="14" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="110" spans="2:4">
+      <c r="B110" s="49" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="112" spans="2:4" ht="18" customHeight="1">
+      <c r="B112" s="48" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="113" spans="2:2">
+      <c r="B113" s="13" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="114" spans="2:2">
+      <c r="B114" s="12" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="115" spans="2:2">
+      <c r="B115" s="14" t="s">
         <v>257</v>
       </c>
     </row>
-    <row r="103" spans="2:2">
-      <c r="B103" s="49" t="s">
+    <row r="116" spans="2:2">
+      <c r="B116" s="49" t="s">
         <v>258</v>
       </c>
     </row>
-    <row r="105" spans="2:2" ht="18" customHeight="1">
-      <c r="B105" s="48" t="s">
+    <row r="118" spans="2:2" ht="18" customHeight="1">
+      <c r="B118" s="48" t="s">
         <v>259</v>
       </c>
     </row>
-    <row r="106" spans="2:2">
-      <c r="B106" s="13" t="s">
+    <row r="119" spans="2:2">
+      <c r="B119" s="13" t="s">
         <v>260</v>
       </c>
     </row>
-    <row r="107" spans="2:2">
-      <c r="B107" s="12" t="s">
+    <row r="120" spans="2:2">
+      <c r="B120" s="12" t="s">
         <v>247</v>
       </c>
     </row>
-    <row r="108" spans="2:2">
-      <c r="B108" s="14" t="s">
+    <row r="121" spans="2:2">
+      <c r="B121" s="14" t="s">
         <v>261</v>
       </c>
     </row>
-    <row r="109" spans="2:2">
-      <c r="B109" s="49" t="s">
+    <row r="122" spans="2:2">
+      <c r="B122" s="49" t="s">
         <v>262</v>
       </c>
     </row>
-    <row r="111" spans="2:2" ht="18" customHeight="1">
-      <c r="B111" s="48" t="s">
+    <row r="124" spans="2:2" ht="18" customHeight="1">
+      <c r="B124" s="48" t="s">
         <v>263</v>
       </c>
     </row>
-    <row r="112" spans="2:2">
-      <c r="B112" s="12" t="s">
+    <row r="125" spans="2:2">
+      <c r="B125" s="12" t="s">
         <v>264</v>
       </c>
     </row>
-    <row r="113" spans="2:2">
-      <c r="B113" s="50" t="s">
+    <row r="126" spans="2:2">
+      <c r="B126" s="50" t="s">
         <v>265</v>
       </c>
     </row>
-    <row r="114" spans="2:2">
-      <c r="B114" s="50" t="s">
+    <row r="127" spans="2:2">
+      <c r="B127" s="50" t="s">
         <v>266</v>
       </c>
     </row>
-    <row r="115" spans="2:2">
-      <c r="B115" s="50" t="s">
+    <row r="128" spans="2:2">
+      <c r="B128" s="50" t="s">
         <v>267</v>
       </c>
     </row>
-    <row r="119" spans="2:2" ht="18" customHeight="1">
-      <c r="B119" s="47" t="s">
+    <row r="132" spans="2:2" ht="18" customHeight="1">
+      <c r="B132" s="47" t="s">
         <v>268</v>
       </c>
     </row>
-    <row r="120" spans="2:2">
-      <c r="B120" t="s">
+    <row r="133" spans="2:2">
+      <c r="B133" t="s">
         <v>269</v>
       </c>
     </row>
-    <row r="121" spans="2:2">
-      <c r="B121" s="1" t="s">
+    <row r="134" spans="2:2">
+      <c r="B134" s="1" t="s">
         <v>270</v>
       </c>
     </row>
-    <row r="122" spans="2:2">
-      <c r="B122" s="1" t="s">
+    <row r="135" spans="2:2">
+      <c r="B135" s="1" t="s">
         <v>271</v>
       </c>
     </row>
-    <row r="123" spans="2:2">
-      <c r="B123" s="1" t="s">
+    <row r="136" spans="2:2">
+      <c r="B136" s="1" t="s">
         <v>272</v>
       </c>
     </row>
-    <row r="124" spans="2:2">
-      <c r="B124" s="1" t="s">
+    <row r="137" spans="2:2">
+      <c r="B137" s="1" t="s">
         <v>273</v>
       </c>
     </row>
-    <row r="125" spans="2:2">
-      <c r="B125" s="1" t="s">
+    <row r="138" spans="2:2">
+      <c r="B138" s="1" t="s">
         <v>274</v>
       </c>
     </row>
@@ -7519,30 +8350,30 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:5" ht="15" customHeight="1">
-      <c r="B2" s="104" t="s">
+      <c r="B2" s="86" t="s">
         <v>631</v>
       </c>
-      <c r="C2" s="103" t="s">
+      <c r="C2" s="85" t="s">
         <v>632</v>
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="B3" s="104" t="s">
+      <c r="B3" s="86" t="s">
         <v>633</v>
       </c>
-      <c r="C3" s="103" t="s">
+      <c r="C3" s="85" t="s">
         <v>634</v>
       </c>
     </row>
-    <row r="4" spans="1:5" s="105" customFormat="1">
-      <c r="B4" s="104" t="s">
+    <row r="4" spans="1:5" s="87" customFormat="1">
+      <c r="B4" s="86" t="s">
         <v>635</v>
       </c>
-      <c r="C4" s="103" t="s">
+      <c r="C4" s="85" t="s">
         <v>636</v>
       </c>
     </row>
-    <row r="5" spans="1:5" s="105" customFormat="1"/>
+    <row r="5" spans="1:5" s="87" customFormat="1"/>
     <row r="6" spans="1:5" ht="15" customHeight="1">
       <c r="A6" t="s">
         <v>275</v>
@@ -7554,15 +8385,15 @@
         <v>276</v>
       </c>
     </row>
-    <row r="7" spans="1:5" s="106" customFormat="1" ht="63">
-      <c r="B7" s="107" t="s">
+    <row r="7" spans="1:5" s="88" customFormat="1" ht="63">
+      <c r="B7" s="89" t="s">
         <v>277</v>
       </c>
       <c r="C7" s="34" t="s">
         <v>278</v>
       </c>
-      <c r="D7" s="107"/>
-      <c r="E7" s="108" t="s">
+      <c r="D7" s="89"/>
+      <c r="E7" s="90" t="s">
         <v>637</v>
       </c>
     </row>
@@ -8615,49 +9446,49 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:36" ht="30" customHeight="1">
-      <c r="A1" s="96" t="s">
+      <c r="A1" s="97" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="97"/>
-      <c r="C1" s="98"/>
-      <c r="D1" s="90"/>
-      <c r="E1" s="90"/>
-      <c r="F1" s="90"/>
-      <c r="G1" s="90"/>
-      <c r="H1" s="90"/>
-      <c r="I1" s="90"/>
-      <c r="J1" s="90"/>
-      <c r="K1" s="90"/>
-      <c r="L1" s="90"/>
-      <c r="M1" s="99"/>
+      <c r="B1" s="98"/>
+      <c r="C1" s="99"/>
+      <c r="D1" s="100"/>
+      <c r="E1" s="100"/>
+      <c r="F1" s="100"/>
+      <c r="G1" s="100"/>
+      <c r="H1" s="100"/>
+      <c r="I1" s="100"/>
+      <c r="J1" s="100"/>
+      <c r="K1" s="100"/>
+      <c r="L1" s="100"/>
+      <c r="M1" s="101"/>
     </row>
     <row r="2" spans="1:36" s="61" customFormat="1" ht="15.95" customHeight="1">
-      <c r="A2" s="102" t="s">
+      <c r="A2" s="105" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="101"/>
-      <c r="C2" s="101"/>
-      <c r="D2" s="100" t="s">
+      <c r="B2" s="104"/>
+      <c r="C2" s="104"/>
+      <c r="D2" s="103" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="101"/>
-      <c r="F2" s="101"/>
-      <c r="G2" s="101"/>
-      <c r="H2" s="101"/>
-      <c r="I2" s="101"/>
-      <c r="J2" s="101"/>
-      <c r="K2" s="101"/>
-      <c r="L2" s="101"/>
-      <c r="M2" s="101"/>
+      <c r="E2" s="104"/>
+      <c r="F2" s="104"/>
+      <c r="G2" s="104"/>
+      <c r="H2" s="104"/>
+      <c r="I2" s="104"/>
+      <c r="J2" s="104"/>
+      <c r="K2" s="104"/>
+      <c r="L2" s="104"/>
+      <c r="M2" s="104"/>
       <c r="N2" s="55"/>
-      <c r="O2" s="94" t="s">
+      <c r="O2" s="106" t="s">
         <v>3</v>
       </c>
-      <c r="P2" s="95"/>
-      <c r="Q2" s="95"/>
-      <c r="R2" s="95"/>
-      <c r="S2" s="95"/>
-      <c r="T2" s="95"/>
+      <c r="P2" s="107"/>
+      <c r="Q2" s="107"/>
+      <c r="R2" s="107"/>
+      <c r="S2" s="107"/>
+      <c r="T2" s="107"/>
       <c r="U2" s="73"/>
       <c r="V2" s="73"/>
       <c r="W2" s="73"/>
@@ -9456,21 +10287,21 @@
       </c>
     </row>
     <row r="15" spans="1:36">
-      <c r="A15" s="88" t="s">
+      <c r="A15" s="102" t="s">
         <v>41</v>
       </c>
-      <c r="B15" s="97"/>
-      <c r="C15" s="98"/>
-      <c r="D15" s="90"/>
-      <c r="E15" s="90"/>
-      <c r="F15" s="90"/>
-      <c r="G15" s="90"/>
-      <c r="H15" s="90"/>
-      <c r="I15" s="90"/>
-      <c r="J15" s="90"/>
-      <c r="K15" s="90"/>
-      <c r="L15" s="90"/>
-      <c r="M15" s="97"/>
+      <c r="B15" s="98"/>
+      <c r="C15" s="99"/>
+      <c r="D15" s="100"/>
+      <c r="E15" s="100"/>
+      <c r="F15" s="100"/>
+      <c r="G15" s="100"/>
+      <c r="H15" s="100"/>
+      <c r="I15" s="100"/>
+      <c r="J15" s="100"/>
+      <c r="K15" s="100"/>
+      <c r="L15" s="100"/>
+      <c r="M15" s="98"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -9501,47 +10332,47 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="30" customHeight="1">
-      <c r="A1" s="93" t="s">
+      <c r="A1" s="114" t="s">
         <v>473</v>
       </c>
-      <c r="B1" s="89"/>
-      <c r="C1" s="90"/>
-      <c r="D1" s="91"/>
-      <c r="E1" s="90"/>
-      <c r="F1" s="90"/>
-      <c r="G1" s="90"/>
-      <c r="H1" s="90"/>
-      <c r="I1" s="90"/>
-      <c r="J1" s="90"/>
-      <c r="K1" s="90"/>
-      <c r="L1" s="90"/>
-      <c r="M1" s="90"/>
+      <c r="B1" s="111"/>
+      <c r="C1" s="100"/>
+      <c r="D1" s="112"/>
+      <c r="E1" s="100"/>
+      <c r="F1" s="100"/>
+      <c r="G1" s="100"/>
+      <c r="H1" s="100"/>
+      <c r="I1" s="100"/>
+      <c r="J1" s="100"/>
+      <c r="K1" s="100"/>
+      <c r="L1" s="100"/>
+      <c r="M1" s="100"/>
     </row>
     <row r="2" spans="1:20" ht="15.95" customHeight="1">
-      <c r="A2" s="92" t="s">
+      <c r="A2" s="113" t="s">
         <v>474</v>
       </c>
-      <c r="B2" s="87"/>
+      <c r="B2" s="110"/>
       <c r="C2" s="56"/>
-      <c r="D2" s="85" t="s">
+      <c r="D2" s="108" t="s">
         <v>475</v>
       </c>
-      <c r="E2" s="86"/>
-      <c r="F2" s="86"/>
-      <c r="G2" s="86"/>
-      <c r="H2" s="86"/>
-      <c r="I2" s="86"/>
-      <c r="J2" s="86"/>
-      <c r="K2" s="86"/>
-      <c r="L2" s="87"/>
-      <c r="O2" s="94" t="s">
+      <c r="E2" s="109"/>
+      <c r="F2" s="109"/>
+      <c r="G2" s="109"/>
+      <c r="H2" s="109"/>
+      <c r="I2" s="109"/>
+      <c r="J2" s="109"/>
+      <c r="K2" s="109"/>
+      <c r="L2" s="110"/>
+      <c r="O2" s="106" t="s">
         <v>3</v>
       </c>
-      <c r="P2" s="95"/>
-      <c r="Q2" s="95"/>
-      <c r="R2" s="95"/>
-      <c r="S2" s="95"/>
-      <c r="T2" s="95"/>
+      <c r="P2" s="107"/>
+      <c r="Q2" s="107"/>
+      <c r="R2" s="107"/>
+      <c r="S2" s="107"/>
+      <c r="T2" s="107"/>
     </row>
     <row r="3" spans="1:20" ht="36" customHeight="1">
       <c r="A3" s="62" t="s">
@@ -10073,21 +10904,21 @@
       <c r="L12" s="75"/>
     </row>
     <row r="13" spans="1:20" ht="12.95" customHeight="1">
-      <c r="A13" s="88" t="s">
+      <c r="A13" s="102" t="s">
         <v>504</v>
       </c>
-      <c r="B13" s="89"/>
-      <c r="C13" s="90"/>
-      <c r="D13" s="91"/>
-      <c r="E13" s="90"/>
-      <c r="F13" s="90"/>
-      <c r="G13" s="90"/>
-      <c r="H13" s="90"/>
-      <c r="I13" s="90"/>
-      <c r="J13" s="90"/>
-      <c r="K13" s="90"/>
-      <c r="L13" s="90"/>
-      <c r="M13" s="90"/>
+      <c r="B13" s="111"/>
+      <c r="C13" s="100"/>
+      <c r="D13" s="112"/>
+      <c r="E13" s="100"/>
+      <c r="F13" s="100"/>
+      <c r="G13" s="100"/>
+      <c r="H13" s="100"/>
+      <c r="I13" s="100"/>
+      <c r="J13" s="100"/>
+      <c r="K13" s="100"/>
+      <c r="L13" s="100"/>
+      <c r="M13" s="100"/>
     </row>
     <row r="14" spans="1:20" ht="29.25" customHeight="1">
       <c r="A14" s="75"/>

</xml_diff>